<commit_message>
Add Final Source for SHIP_FROM_ORG and UOM
Set column G (Final Source) for rows 12 (SHIP_FROM_ORG) and 14 (UOM)
to their DOO_FULFILL_LINES_ALL source columns.

https://claude.ai/code/session_01V2jE9rtLxf7pmmyHXZav2o
</commit_message>
<xml_diff>
--- a/fact_Service_metrics dates analysis1.xlsx
+++ b/fact_Service_metrics dates analysis1.xlsx
@@ -2930,6 +2930,11 @@
           <t>STG: TRIM(CAST(SQ_BCI_SALES_ORDLNS.SHIP_FROM_ORG_ID AS STRING)) = FulfillLine.FULFILLLINEFULFILLORGID -&gt; INVENTORY_ORG_ID</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
@@ -2987,6 +2992,11 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>TRIM(COALESCE(SQ_BCI_SALES_ORDLNS.ORDER_QUANTITY_UOM, '__UNASSIGNED__')) -&gt; FulfillLine.FULFILLLINEORDEREDUOM</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDUOM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Populate Final Source for all 150 columns in FSM Columns sheet
Filled column G (Final Source) for every row using the NBLBI_FUSION_ONT
schema prefix. Maps each FSM column to its ultimate source:
- DOO_HEADERS_ALL / DOO_LINES_ALL / DOO_FULFILL_LINES_ALL columns
- HZ_CUST_SITE_USES_ALL ship-to lookups via DIM_CUST_SITE_USE
- DIM_INV_MASTER_ITEMS item attributes via INVENTORY_ITEM_ID + SHIP_FROM_ORG_ID
- DIM_HR_ORG for ship-from / ship-to org attributes
- PLP (Plan Pro - SOLF/plp tables) for SO-only columns
- N/A for derived, hardcoded, dim-lookup, and FACT_ORDER_HISTORY_ACTIVITY rows

https://claude.ai/code/session_01V2jE9rtLxf7pmmyHXZav2o
</commit_message>
<xml_diff>
--- a/fact_Service_metrics dates analysis1.xlsx
+++ b/fact_Service_metrics dates analysis1.xlsx
@@ -2615,7 +2615,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CREATE / UPDATE</t>
+          <t>CREATE / UPDATE (hardcoded literal)</t>
         </is>
       </c>
     </row>
@@ -2645,6 +2645,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>N/A - dim lookup (DIM_MCAL_PLANNING_WEEK on FINAL_PROMISE_DATE_LOCAL)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="9" t="inlineStr">
@@ -2677,6 +2682,11 @@
           <t>PLP</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30.75" customHeight="1">
       <c r="A5" s="9" t="inlineStr">
@@ -2709,6 +2719,11 @@
           <t>PLP</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="45.75" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
@@ -2736,6 +2751,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; SHIP_TO_ORG_ID; PLP - COALESCE(plp1.SK_X_SHIP_TO_ORG_ID, SOLF.SK_X_SHIP_TO_ORG_ID)</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.CUSTOMER_NAME</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30.75" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -2770,7 +2790,7 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>DOO_HEADERS_ALL.HEADERCUSTOMERPONUMBER</t>
+          <t>NBLBI_FUSION_ONT.DOO_HEADERS_ALL.HEADERCUSTOMERPONUMBER</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2827,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>DOO_HEADERS_ALL.HEADERORDERNUMBER</t>
+          <t>NBLBI_FUSION_ONT.DOO_HEADERS_ALL.HEADERORDERNUMBER</t>
         </is>
       </c>
     </row>
@@ -2840,8 +2860,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>DOO_LINES_ALL.LINELINENUMBER and 
-WSH_DELIVERY_DETAILS.DELIVERYLINEPEOSOURCESHIPMENTNUMBER</t>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINELINENUMBER + NBLBI_FUSION_ONT.WSH_DELIVERY_DETAILS.DELIVERYLINEPEOSOURCESHIPMENTNUMBER</t>
         </is>
       </c>
     </row>
@@ -2876,6 +2895,11 @@
           <t>PLP</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="60.75" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
@@ -2903,6 +2927,11 @@
           <t>DOO_HEADERS_ALL.HEADERFREIGHTTERMSCODE</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_HEADERS_ALL.HEADERFREIGHTTERMSCODE</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
@@ -2962,6 +2991,11 @@
           <t>STG: INVENTORY_ITEM_ID-SHIP_FROM_ORG_ID concat = DOO_LINES_ALL.LINEINVENTORYITEMID + SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.PRODUCT_NUM</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
@@ -3026,6 +3060,11 @@
           <t>STG: SQ_BCI_SALES_ORDLNS.ORDERED_QUANTITY AS SALES_QTY -&gt; FulfillLine.FULFILLLINEORDEREDQTY</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
@@ -3053,6 +3092,11 @@
           <t>STG: SALES_QTY = ORDERED_QUANTITY (FulfillLine.FULFILLLINEORDEREDQTY); CONVERSION_RATE from dim</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY * DIM_INV_MASTER_ITEMS.X_ATTRIBUTE5 (24pk conversion)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
@@ -3085,6 +3129,11 @@
           <t>STG: SQ_BCI_SALES_ORDLNS.SHIPPED_QUANTITY -&gt; FulfillLine.FULFILLLINESHIPPEDQTY</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINESHIPPEDQTY</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
@@ -3112,6 +3161,11 @@
           <t>STG: TOTAL_SHIPPED_QTY = SHIPPED_QUANTITY; conversion via DIM_UNIT_OF_MEASURE_D</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINESHIPPEDQTY * DIM_INV_MASTER_ITEMS.X_ATTRIBUTE5 (24pk conversion)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -3139,6 +3193,11 @@
           <t>STG: ORDERED_QUANTITY - SHIPPED_QUANTITY (FulfillLine columns)</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY - FULFILLLINESHIPPEDQTY</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
@@ -3166,6 +3225,11 @@
           <t>STG: ORDERED_QUANTITY - SHIPPED_QUANTITY</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY - FULFILLLINESHIPPEDQTY) * DIM_INV_MASTER_ITEMS.X_ATTRIBUTE5</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
@@ -3193,6 +3257,11 @@
           <t>STG: TRIM(SQ_BCI_SALES_ORDLNS.OLA_ATTRIBUTE7) -&gt; FulfillLine attribute (DOO_FULFILL_LINES extension)</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_EFF.OLA_ATTRIBUTE7 (FulfillLine extension)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
@@ -3220,6 +3289,11 @@
           <t>N/A - sourced from FACT_ORDER_HISTORY_ACTIVITY</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>N/A - sourced from FACT_ORDER_HISTORY_ACTIVITY</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
@@ -3252,6 +3326,11 @@
           <t>STG: TRIM(SQ_BCI_SALES_ORDLNS.OLA_ATTRIBUTE12) - DOO_FULFILL_LINES_EFF attribute</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_EFF.OLA_ATTRIBUTE12</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
@@ -3279,6 +3358,11 @@
           <t>STG: 'SALES_ORDER_PROCESS-'||FLOW_STATUS_CODE1 -&gt; X_ORDER_LINE_STATUS_ID (FulfillLine.FULFILLLINESTATUSCODE)</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINESTATUSCODE -&gt; DIM_OM_LINE_STATUS</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
@@ -3306,6 +3390,11 @@
           <t>N/A - sourced from FACT_ORDER_HISTORY_ACTIVITY</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>N/A - sourced from FACT_ORDER_HISTORY_ACTIVITY</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
@@ -3333,6 +3422,11 @@
           <t>N/A - sourced from FACT_ORDER_HISTORY_ACTIVITY</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>N/A - sourced from FACT_ORDER_HISTORY_ACTIVITY</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
@@ -3365,6 +3459,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; SHIP_TO_ORG_ID</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.CITY_CODE</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
@@ -3397,6 +3496,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.STATEPROVINCE_CODE</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
@@ -3424,6 +3528,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.POSTAL_CODE</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
@@ -3456,6 +3565,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.PARTY_SITE_NUMBER</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
@@ -3488,6 +3602,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.DISTRIBUTION_CHANNEL_CODE</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
@@ -3520,6 +3639,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.DSD</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
@@ -3547,6 +3671,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Derived from NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.DSD + DISTRIBUTION_CHANNEL_CODE (DECODE)</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
@@ -3579,6 +3708,11 @@
           <t>PLP - COALESCE(plp4.CARRIER_NAME, SOLF.CARRIER_NAME); STG sets CARRIER_NAME = NULL</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
@@ -3611,6 +3745,11 @@
           <t>PLP - COALESCE(plp2.SHIPMENT_GID, SOLF.SHIPMENT_GID); STG sets SHIPMENT_GID = NULL</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
@@ -3638,6 +3777,11 @@
           <t>STG: 'SALES_CYCLE_HEADER_PROCESS-'||HEADER_FLOW_STATUS_CODE -&gt; HEADER_STATUS_ID (DOO_HEADERS_ALL.HEADERSTATUSCODE)</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_HEADERS_ALL.HEADERSTATUSCODE -&gt; DIM_OM_STATUS</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
@@ -3665,6 +3809,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_BOTTLE_SIZE</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
@@ -3692,6 +3841,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_PACK_SIZE</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
@@ -3719,6 +3873,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_PRODUCT</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
@@ -3746,6 +3905,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_PRODUCT_FAMILY</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
@@ -3773,6 +3937,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_PRODUCT_CATEGORY</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
@@ -3800,6 +3969,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_PRODUCT_CATEGORY_SC</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
@@ -3827,6 +4001,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_FG_SALES_CATGORY (DECODE with X_PRODUCT when PRODUCT_TYPE_CODE=SA)</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
@@ -3854,6 +4033,11 @@
           <t>N/A - sourced from FACT_ORDER_HISTORY_ACTIVITY</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>N/A - sourced from FACT_ORDER_HISTORY_ACTIVITY</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
@@ -3886,6 +4070,11 @@
           <t>PLP - COALESCE(plp3.OR_TRANSPORT_MODE_GID, plp2.OR_TRANSPORT_MODE_GID, SOLF.OR_TRANSPORT_MODE_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
@@ -3913,6 +4102,11 @@
           <t>PLP - COALESCE(plp4.SH_TRANSPORT_MODE_GID, SOLF.SH_TRANSPORT_MODE_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
@@ -3940,6 +4134,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="9" t="inlineStr">
@@ -3967,6 +4166,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
@@ -3994,6 +4198,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="9" t="inlineStr">
@@ -4021,6 +4230,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
@@ -4048,6 +4262,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="9" t="inlineStr">
@@ -4075,6 +4294,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
@@ -4102,6 +4326,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="9" t="inlineStr">
@@ -4129,6 +4358,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
@@ -4156,6 +4390,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="9" t="inlineStr">
@@ -4183,6 +4422,11 @@
           <t>N/A - hardcoded in FSM</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>N/A - hardcoded literal in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="9" t="inlineStr">
@@ -4210,6 +4454,11 @@
           <t>STG: FulfillLine.FULFILLLINEFULFILLORGID -&gt; INVENTORY_ORG_ID</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_HR_ORG.X_ROLLUP_ORGANIZATION_CODE</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="9" t="inlineStr">
@@ -4237,6 +4486,11 @@
           <t>STG: FulfillLine.FULFILLLINEFULFILLORGID</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_HR_ORG.X_SUPPLY_CHAIN_REGION</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="9" t="inlineStr">
@@ -4264,6 +4518,11 @@
           <t>STG: derived via DIM_HR_ORG dim lookup</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_HR_ORG -&gt; X_OPERATING_UNIT (DECODE to NBL/NBL-MX)</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="9" t="inlineStr">
@@ -4296,6 +4555,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.COUNTRY_CODE</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
@@ -4323,6 +4587,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="9" t="inlineStr">
@@ -4350,6 +4619,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
@@ -4377,6 +4651,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.SITE_USE_ATTRIBUTE18</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="9" t="inlineStr">
@@ -4404,6 +4683,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.NEW_ORGANIC_CUSTOMER</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="9" t="inlineStr">
@@ -4431,6 +4715,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.CUSTOMER_REGION</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="9" t="inlineStr">
@@ -4458,6 +4747,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.LOCATION_GID</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
@@ -4485,6 +4779,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>N/A - dim lookup (DIM_MCAL_PLANNING_WEEK on FINAL_CUSTOMER_AGREED_TO_DATE)</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
@@ -4517,6 +4816,11 @@
           <t>STG: INVENTORY_ITEM_ID-SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_DEPLOYMENT_FLAG</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="9" t="inlineStr">
@@ -4544,6 +4848,11 @@
           <t>STG: SALES_QTY = ORDERED_QUANTITY (FulfillLine.FULFILLLINEORDEREDQTY)</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY (UOM conversion to cases)</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="9" t="inlineStr">
@@ -4571,6 +4880,11 @@
           <t>STG: TOTAL_SHIPPED_QTY = SHIPPED_QUANTITY</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINESHIPPEDQTY (UOM conversion to cases)</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="9" t="inlineStr">
@@ -4598,6 +4912,11 @@
           <t>STG: ORDERED_QUANTITY - SHIPPED_QUANTITY</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>(NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY - FULFILLLINESHIPPEDQTY) (UOM conversion to cases)</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="9" t="inlineStr">
@@ -4625,6 +4944,11 @@
           <t>STG: FulfillLine.FULFILLLINEFULFILLORGID</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_HR_ORG.X_SHIPPING_REGION</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="9" t="inlineStr">
@@ -4652,6 +4976,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.SITE_USE_ATTRIBUTE3</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="9" t="inlineStr">
@@ -4684,6 +5013,11 @@
           <t>PLP - COALESCE(plp2.OR_USER_DEFINED3_ICON_GID, SOLF.OR_USER_DEFINED3_ICON_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="9" t="inlineStr">
@@ -4711,6 +5045,11 @@
           <t>N/A - hardcoded NULL</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>N/A - hardcoded NULL in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="9" t="inlineStr">
@@ -4743,6 +5082,11 @@
           <t>PLP - COALESCE(plp8.STATUS_VALUE_GID, SOLF.STATUS_VALUE_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="9" t="inlineStr">
@@ -4770,6 +5114,11 @@
           <t>STG: X_SALES_STATE_ID derivation</t>
         </is>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Derived via DIM_SALES_STATE on X_SALES_STATE_ID</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="9" t="inlineStr">
@@ -4802,6 +5151,11 @@
           <t>PLP - COALESCE(plp2.OR_RATE_OFFERING_GID, SOLF.OR_RATE_OFFERING_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="9" t="inlineStr">
@@ -4834,6 +5188,11 @@
           <t>PLP - COALESCE(plp2.OR_INDICATOR, SOLF.OR_INDICATOR); STG = NULL</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="9" t="inlineStr">
@@ -4861,6 +5220,11 @@
           <t>STG: CASE WHEN X_REQUEST_DATE IS NULL THEN -2 ELSE DIM_MCAL_PLNG_WK_D_REQ.ROW_WID (joined on date_format(X_REQUEST_DATE))</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>N/A - dim lookup (DIM_MCAL_PLANNING_WEEK on X_REQUEST_DATE)</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="9" t="inlineStr">
@@ -4888,6 +5252,11 @@
           <t>STG: joined on X_REQUEST_DATE</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>N/A - dim lookup (DIM_MCAL_PLANNING_WEEK on X_REQUEST_DATE)</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="9" t="inlineStr">
@@ -4915,6 +5284,11 @@
           <t>PLP - COALESCE(plp2.OR_RATE_GEO_GID, SOLF.OR_RATE_GEO_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="9" t="inlineStr">
@@ -4947,6 +5321,11 @@
           <t>PLP - COALESCE(plp3.X_LANE_GID, SOLF.X_LANE_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="9" t="inlineStr">
@@ -4974,6 +5353,11 @@
           <t>PLP - COALESCE(plp3/plp2.OR_TRANSPORT_MODE_GID, SOLF.OR_TRANSPORT_MODE_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="9" t="inlineStr">
@@ -5006,6 +5390,11 @@
           <t>PLP - COALESCE(plp2.DEPLOYMENT_FLAG, SOLF.DEPLOYMENT_FLAG); STG = NULL</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="9" t="inlineStr">
@@ -5033,6 +5422,11 @@
           <t>PLP - COALESCE(plp4.FINAL_MILES, SOLF.FINAL_MILES); STG = NULL/derived via dim</t>
         </is>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables) / DIM_PLANT_TO_CUSTOMER_MILES.FINAL_MILES</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="9" t="inlineStr">
@@ -5060,6 +5454,11 @@
           <t>PLP - COALESCE(plp2.OR_PENDING_REASON, SOLF.OR_PENDING_REASON); STG = NULL</t>
         </is>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="9" t="inlineStr">
@@ -5092,6 +5491,11 @@
           <t>PLP - COALESCE(plp4.SH_RATE_OFFERING_GID, SOLF.SH_RATE_OFFERING_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="9" t="inlineStr">
@@ -5124,6 +5528,11 @@
           <t>PLP - COALESCE(plp4.SH_RATE_GEO_GID, SOLF.SH_RATE_GEO_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="9" t="inlineStr">
@@ -5151,6 +5560,11 @@
           <t>PLP - COALESCE(plp3.X_LANE_GID, SOLF.X_LANE_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="9" t="inlineStr">
@@ -5183,6 +5597,11 @@
           <t>PLP - COALESCE(plp4.SH_TRANSPORT_MODE_GID, SOLF.SH_TRANSPORT_MODE_GID); STG = NULL</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="9" t="inlineStr">
@@ -5210,6 +5629,11 @@
           <t>STG: SQ_BCI_SALES_ORDLNS.CANCELLED_QUANTITY -&gt; FulfillLine.FULFILLLINECANCELEDQTY</t>
         </is>
       </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINECANCELEDQTY</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="9" t="inlineStr">
@@ -5237,6 +5661,11 @@
           <t>STG: FULFILLLINECANCELEDQTY</t>
         </is>
       </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINECANCELEDQTY * DIM_INV_MASTER_ITEMS.X_ATTRIBUTE5</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="9" t="inlineStr">
@@ -5269,6 +5698,11 @@
           <t>PLP - COALESCE(plp2.SCHEDULE_UPDATE_USER, SOLF.SCHEDULE_UPDATE_USER); STG = NULL</t>
         </is>
       </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="9" t="inlineStr">
@@ -5296,6 +5730,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="9" t="inlineStr">
@@ -5323,6 +5762,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>N/A - derived in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="9" t="inlineStr">
@@ -5350,6 +5794,11 @@
           <t>PLP - COALESCE(plp2.CPU_CONTACT, SOLF.CPU_CONTACT); STG = NULL. Note: FSM uses literal NULL.</t>
         </is>
       </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>N/A - hardcoded NULL in FSM (PLP source CPU_CONTACT ignored)</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="9" t="inlineStr">
@@ -5377,6 +5826,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.ADDRESS</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="9" t="inlineStr">
@@ -5409,6 +5863,11 @@
           <t>PLP - COALESCE(plp4.DOCK_DOOR, SOLF.DOCK_DOOR); STG = NULL</t>
         </is>
       </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="9" t="inlineStr">
@@ -5436,6 +5895,11 @@
           <t>PLP - COALESCE(plp4.LOAD_TYPE, SOLF.LOAD_TYPE) and COALESCE(plp4.LOADTYPE, SOLF.LOADTYPE); STG = NULL</t>
         </is>
       </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="9" t="inlineStr">
@@ -5463,6 +5927,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_FG_BRAND (DECODE with X_PRODUCT_FAMILY when PRODUCT_TYPE_CODE=SA)</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="9" t="inlineStr">
@@ -5490,6 +5959,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_WATER_TYPE</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="9" t="inlineStr">
@@ -5517,6 +5991,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_FG_FLAVOR (DECODE with X_WATER_TYPE when PRODUCT_TYPE_CODE=SA)</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="9" t="inlineStr">
@@ -5544,6 +6023,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_FG_SALES_CATGORY (DECODE with X_PRODUCT when PRODUCT_TYPE_CODE=SA)</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="15.75" customHeight="1">
       <c r="A105" s="9" t="inlineStr">
@@ -5571,6 +6055,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_FG_BUSINESS_UNIT (DECODE with X_ATTRIBUTE14 when PRODUCT_TYPE_CODE=SA)</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="9" t="inlineStr">
@@ -5598,6 +6087,11 @@
           <t>PLP - SOLF.DEF_ORG; STG = NULL. FSM ignores it.</t>
         </is>
       </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>N/A - hardcoded NULL in FSM</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="15.75" customHeight="1">
       <c r="A107" s="9" t="inlineStr">
@@ -5625,6 +6119,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_CUSTOMER_ITEM_NUMBER</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="9" t="inlineStr">
@@ -5657,6 +6156,11 @@
           <t>STG: SOLF.DEF_ROLLUP_ORG_CODE (no PLP override). Likely from DOO/FulfillLine attribute.</t>
         </is>
       </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.DEF_ROLLUP_ORG_CODE (FulfillLine extension)</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="9" t="inlineStr">
@@ -5684,6 +6188,11 @@
           <t>STG: 'SALES_ORDLNS-'||LINE_CATEGORY_CODE||'-'||ORDER_TYPE_ID||'-SELF SHIP/DROP SHIP' -&gt; XACT_TYPE_ID; ORDER_TYPE_ID = DOO_HEADERS_ALL.HEADERORDERTYPECODE</t>
         </is>
       </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_HEADERS_ALL.HEADERORDERTYPECODE -&gt; DIM_OM_TRANSACTION_TYPE.XACT_SUBTYPE_CODE</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="15.75" customHeight="1">
       <c r="A110" s="9" t="inlineStr">
@@ -5711,6 +6220,11 @@
           <t>PLP - COALESCE(plp1.SK_X_DESTINATION_ORGANIZATION_ID, SOLF.SK_X_DESTINATION_ORGANIZATION_ID); STG: DESTINATION_ORGANIZATION_ID</t>
         </is>
       </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEDESTINATIONORGID -&gt; DIM_HR_ORG (PLP override via plp1).ORGANIZATION_CODE</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="9" t="inlineStr">
@@ -5738,6 +6252,11 @@
           <t>PLP - COALESCE(plp1, SOLF) for SK_X_DESTINATION_ORGANIZATION_ID</t>
         </is>
       </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEDESTINATIONORGID -&gt; DIM_HR_ORG (PLP override via plp1).X_ROLLUP_ORGANIZATION_CODE</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="9" t="inlineStr">
@@ -5765,6 +6284,11 @@
           <t>PLP - COALESCE(plp1, SOLF) for SK_X_DESTINATION_ORGANIZATION_ID</t>
         </is>
       </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEDESTINATIONORGID -&gt; DIM_HR_ORG (PLP override via plp1).X_SUPPLY_CHAIN_REGION</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="9" t="inlineStr">
@@ -5792,6 +6316,11 @@
           <t>N/A - derived in FSM</t>
         </is>
       </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>N/A - sourced from FACT_ORDER_HISTORY_ACTIVITY</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="9" t="inlineStr">
@@ -5819,6 +6348,11 @@
           <t>STG: INVENTORY_ITEM_ID-SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_ITEM_DESCRIPTION</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="15.75" customHeight="1">
       <c r="A115" s="9" t="inlineStr">
@@ -5846,6 +6380,11 @@
           <t>N/A - dim lookup in view</t>
         </is>
       </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>N/A - dim lookup (DIM_MCAL_DAY on SHIP_CONFIRM_DATE)</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="9" t="inlineStr">
@@ -5873,6 +6412,11 @@
           <t>N/A - dim lookup in view</t>
         </is>
       </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>N/A - dim lookup (DIM_MCAL_DAY on SHIP_CONFIRM_DATE)</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="9" t="inlineStr">
@@ -5905,6 +6449,11 @@
           <t>STG: HZ_CUST_SITE_USES_ALL.SITEUSEID</t>
         </is>
       </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.HZ_CUST_SITE_USES_ALL.SITEUSEID -&gt; DIM_CUST_SITE_USE.ADDRESS_DESCRIPTION</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="9" t="inlineStr">
@@ -5932,6 +6481,11 @@
           <t>N/A - dim lookup in view</t>
         </is>
       </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>N/A - dim lookup (DIM_MCAL_DAY on SOA_SHIPMENT_DATE)</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="9" t="inlineStr">
@@ -5959,6 +6513,11 @@
           <t>N/A - dim lookup in view</t>
         </is>
       </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>N/A - dim lookup (DIM_MCAL_DAY on SOA_SHIPMENT_DATE)</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="9" t="inlineStr">
@@ -5986,6 +6545,11 @@
           <t>PLP - SOA_SHIPPED_QUANTITY from plp6/plp5/SOLF; STG SOA_SHIPPED_QUANTITY = 0</t>
         </is>
       </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables) - SOA_SHIPPED_QUANTITY (derived: QTY_REQUESTED - SOA_SHIPPED_QUANTITY)</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="9" t="inlineStr">
@@ -6013,6 +6577,11 @@
           <t>PLP - SOA_SHIPPED_QUANTITY from plp6/plp5</t>
         </is>
       </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables) - SOA_SHIPPED_QUANTITY * DIM_INV_MASTER_ITEMS.X_ATTRIBUTE5 (capped at PKEQ24_CASES_REQUESTED)</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="15.75" customHeight="1">
       <c r="A122" s="9" t="inlineStr">
@@ -6040,6 +6609,11 @@
           <t>PLP for SOA_SHIPPED_QUANTITY</t>
         </is>
       </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables) - SOA_SHIPPED_QUANTITY (derived * X_ATTRIBUTE5)</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="9" t="inlineStr">
@@ -6067,6 +6641,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_ATTRIBUTE14</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="9" t="inlineStr">
@@ -6094,6 +6673,11 @@
           <t>STG: ORDERED_QTY = ORDERED_QUANTITY + CANCELLED_QUANTITY from FulfillLine</t>
         </is>
       </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY + FULFILLLINECANCELEDQTY (UOM conversion, FIRST_VALUE window)</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="9" t="inlineStr">
@@ -6121,6 +6705,11 @@
           <t>STG: ORDERED_QTY (FulfillLine.FULFILLLINEORDEREDQTY + CANCELLED)</t>
         </is>
       </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>(NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY + FULFILLLINECANCELEDQTY) * DIM_INV_MASTER_ITEMS.X_ATTRIBUTE5</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="9" t="inlineStr">
@@ -6148,6 +6737,11 @@
           <t>PLP - COALESCE(plp1.SK_X_DESTINATION_ORGANIZATION_ID, SOLF.SK_X_DESTINATION_ORGANIZATION_ID)</t>
         </is>
       </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEDESTINATIONORGID -&gt; DIM_HR_ORG (PLP override via plp1).X_SHIPPING_REGION</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="15.75" customHeight="1">
       <c r="A127" s="9" t="inlineStr">
@@ -6175,6 +6769,11 @@
           <t>PLP - COALESCE(plp4.SUPPLY_CHAIN_LOADTYPE, SOLF.SUPPLY_CHAIN_LOADTYPE); STG = NULL</t>
         </is>
       </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="9" t="inlineStr">
@@ -6202,6 +6801,11 @@
           <t>N/A - derived in view</t>
         </is>
       </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>N/A - derived in view from STATUS + CANCEL_REASON_CODE (CASE)</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="9" t="inlineStr">
@@ -6229,6 +6833,11 @@
           <t>STG: SALES_QTY = ORDERED_QUANTITY (FulfillLine)</t>
         </is>
       </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY (UOM conversion to pallets)</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="15.75" customHeight="1">
       <c r="A130" s="9" t="inlineStr">
@@ -6256,6 +6865,11 @@
           <t>STG: TOTAL_SHIPPED_QTY = SHIPPED_QUANTITY (FulfillLine)</t>
         </is>
       </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINESHIPPEDQTY (UOM conversion to pallets)</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="15.75" customHeight="1">
       <c r="A131" s="9" t="inlineStr">
@@ -6283,6 +6897,11 @@
           <t>STG: ORDERED_QUANTITY - SHIPPED_QUANTITY</t>
         </is>
       </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>(NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY - FULFILLLINESHIPPEDQTY) (UOM conversion to pallets)</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="15.75" customHeight="1">
       <c r="A132" s="9" t="inlineStr">
@@ -6310,6 +6929,11 @@
           <t>STG: CANCELLED_QTY = SQ_BCI_SALES_ORDLNS.CANCELLED_QUANTITY = FulfillLine.FULFILLLINECANCELEDQTY</t>
         </is>
       </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINECANCELEDQTY (UOM conversion to cases)</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="9" t="inlineStr">
@@ -6337,6 +6961,11 @@
           <t>STG: CANCELLED_QTY from FulfillLine.FULFILLLINECANCELEDQTY</t>
         </is>
       </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINECANCELEDQTY (UOM conversion to 24pk)</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="9" t="inlineStr">
@@ -6364,6 +6993,11 @@
           <t>STG: CANCELLED_QTY from FulfillLine.FULFILLLINECANCELEDQTY</t>
         </is>
       </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINECANCELEDQTY (UOM conversion to pallets)</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="15.75" customHeight="1">
       <c r="A135" s="9" t="inlineStr">
@@ -6391,6 +7025,11 @@
           <t>STG: ORDERED_QUANTITY - SHIPPED_QUANTITY</t>
         </is>
       </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>(NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEORDEREDQTY - FULFILLLINESHIPPEDQTY) * DIM_INV_MASTER_ITEMS.X_ATTRIBUTE5</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="15.75" customHeight="1">
       <c r="A136" s="9" t="inlineStr">
@@ -6423,6 +7062,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_WATER_TYPE_SC</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="15.75" customHeight="1">
       <c r="A137" s="9" t="inlineStr">
@@ -6450,6 +7094,11 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>N/A - dim lookup (DIM_MCAL_PLANNING_WEEK on FINAL_CUSTOMER_AGREED_TO_DATE)</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="9" t="inlineStr">
@@ -6482,6 +7131,11 @@
           <t>STG: TRIM(SQ_BCI_SALES_ORDLNS.X_SHIPMENT_PRIORITY_CODE) - DOO/FulfillLine attribute</t>
         </is>
       </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_EFF.X_SHIPMENT_PRIORITY_CODE</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="9" t="inlineStr">
@@ -6514,6 +7168,11 @@
           <t>STG: TRIM(SQ_BCI_SALES_ORDLNS.X_OLA_DEMAND_CLASS_CODE) - DOO/FulfillLine attribute</t>
         </is>
       </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_EFF.X_OLA_DEMAND_CLASS_CODE (UPDATE from OHA.OLH_DEMAND_CLASS_CODE)</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="15.75" customHeight="1">
       <c r="A140" s="9" t="inlineStr">
@@ -6541,6 +7200,11 @@
           <t>STG: TRIM(SQ_BCI_SALES_ORDLNS.OLA_ATTRIBUTE13) - DOO/FulfillLine attribute</t>
         </is>
       </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_EFF.OLA_ATTRIBUTE13 (UPDATE from OHA.ATTRIBUTE13)</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="15.75" customHeight="1">
       <c r="A141" s="9" t="inlineStr">
@@ -6568,6 +7232,11 @@
           <t>STG: TRIM(SQ_BCI_SALES_ORDLNS.OLA_ATTRIBUTE14) - DOO/FulfillLine attribute</t>
         </is>
       </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_EFF.OLA_ATTRIBUTE14 (UPDATE from OHA.ATTRIBUTE14)</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="15.75" customHeight="1">
       <c r="A142" s="9" t="inlineStr">
@@ -6600,6 +7269,11 @@
           <t>PLP - COALESCE(plp4.SHIPMENT_PRELOAD, SOLF.SHIPMENT_PRELOAD); STG = NULL</t>
         </is>
       </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="9" t="inlineStr">
@@ -6627,6 +7301,11 @@
           <t>PLP - COALESCE(plp6.SOA_SHIPPED_QUANTITY, plp5.SOA_SHIPPED_QUANTITY, SOLF.SOA_SHIPPED_QUANTITY); STG SOA_SHIPPED_QUANTITY = 0</t>
         </is>
       </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables) - SOA_SHIPPED_QUANTITY (capped at FULFILLLINEORDEREDQTY)</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="9" t="inlineStr">
@@ -6659,6 +7338,11 @@
           <t>PLP - COALESCE(plp2.OREF_SCHEDULE_INSERT_USER, SOLF.OREF_SCHEDULE_INSERT_USER); STG = NULL</t>
         </is>
       </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="15.75" customHeight="1">
       <c r="A145" s="9" t="inlineStr">
@@ -6691,6 +7375,11 @@
           <t>PLP - COALESCE(plp2.WITH_DRAW_USER_FLAG, SOLF.WITH_DRAW_USER_FLAG); STG = NULL</t>
         </is>
       </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="15.75" customHeight="1">
       <c r="A146" s="9" t="inlineStr">
@@ -6718,6 +7407,11 @@
           <t>STG: FulfillLine quantities</t>
         </is>
       </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>N/A - derived in view (ORIGINAL_REQUESTED_QTY - ACTUAL_CASES_REQUESTED)</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="15.75" customHeight="1">
       <c r="A147" s="9" t="inlineStr">
@@ -6745,6 +7439,11 @@
           <t>STG: INVENTORY_ITEM_ID - SHIP_FROM_ORG_ID</t>
         </is>
       </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_LINES_ALL.LINEINVENTORYITEMID + NBLBI_FUSION_ONT.DOO_FULFILL_LINES_ALL.FULFILLLINEFULFILLORGID -&gt; DIM_INV_MASTER_ITEMS.X_ATTRIBUTE14</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="9" t="inlineStr">
@@ -6772,6 +7471,11 @@
           <t>PLP - COALESCE(plp1.X_OLA_ATTRIBUTE16, SOLF.X_OLA_ATTRIBUTE16); STG: SQ_BCI_SALES_ORDLNS.X_OLA_ATTRIBUTE16</t>
         </is>
       </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>NBLBI_FUSION_ONT.DOO_FULFILL_LINES_EFF.OLA_ATTRIBUTE16 (DECODE = MTO -&gt; 1)</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="15.75" customHeight="1">
       <c r="A149" s="9" t="inlineStr">
@@ -6804,6 +7508,11 @@
           <t>PLP - COALESCE(plp2.SK_OSP_ID, -1); STG = -2 (cast as BIGINT). Actual values from PLP.</t>
         </is>
       </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables) - SK_OSP_ID</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="15.75" customHeight="1">
       <c r="A150" s="9" t="inlineStr">
@@ -6836,6 +7545,11 @@
           <t>PLP - COALESCE(plp2.SK_MOSP_ID, -1); STG default. Actual values from PLP.</t>
         </is>
       </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>PLP (Plan Pro - SOLF/plp tables) - SK_MOSP_ID</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="15.75" customHeight="1">
       <c r="A151" s="9" t="inlineStr">
@@ -6861,6 +7575,11 @@
       <c r="F151" t="inlineStr">
         <is>
           <t>N/A - derived in FSM</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>N/A - sourced from FACT_ORDER_HISTORY_ACTIVITY</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expand PLP shorthand to specific NBLBI_PLP table.column in column G
Replaced generic "PLP (Plan Pro - SOLF/plp tables)" entries with the
exact NBLBI_PLP source table and column (e.g.,
SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.TRIP_ID,
SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.CARRIER_NAME,
FACT_SALES_ORDERLINE_SOASHIPPEDQUANTITY_PLP.SOA_SHIPPED_QUANTITY, etc.)
based on the join mapping in fact_sales_order_line.py.

https://claude.ai/code/session_01V2jE9rtLxf7pmmyHXZav2o
</commit_message>
<xml_diff>
--- a/fact_Service_metrics dates analysis1.xlsx
+++ b/fact_Service_metrics dates analysis1.xlsx
@@ -2684,7 +2684,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.TRIP_ID</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.STOP_NUMBER (MAX per trip)</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_ORDER_STG.FACT_SALES_ORDER_LINE_STG.DELIVERY_ID (carryover from prior SOLF)</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.CARRIER_NAME</t>
         </is>
       </c>
     </row>
@@ -3747,7 +3747,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.SHIPMENT_GID</t>
         </is>
       </c>
     </row>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.SH_TRANSPORT_MODE_GID (also stored on SOLF as TRANSPORT_MODE_GID)</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>Derived from NBLBI_PLP.SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.SH_TRANSPORT_MODE_GID = 'NBL.DROP'</t>
         </is>
       </c>
     </row>
@@ -5015,7 +5015,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.OR_SCHEDULE_FLAG</t>
         </is>
       </c>
     </row>
@@ -5084,7 +5084,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_STATUS_UPDATE_PLP.STATUS_VALUE_GID</t>
         </is>
       </c>
     </row>
@@ -5153,7 +5153,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.OR_RATE_OFFERING_GID</t>
         </is>
       </c>
     </row>
@@ -5190,7 +5190,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.OR_INDICATOR</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.OR_RATE_GEO_GID</t>
         </is>
       </c>
     </row>
@@ -5323,7 +5323,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_XLANE_UPDATE.X_LANE_GID (Sales History variant SH_X_LANE_GID)</t>
         </is>
       </c>
     </row>
@@ -5355,7 +5355,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.OR_TRANSPORT_MODE_GID</t>
         </is>
       </c>
     </row>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.OR_DEPLOYMENT_FLAG</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5424,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables) / DIM_PLANT_TO_CUSTOMER_MILES.FINAL_MILES</t>
+          <t>DIM_PLANT_TO_CUSTOMER_MILES.FINAL_MILES (joined on SHIP_FROM_ORG + SHIP_TO_PARTY_SITE)</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5456,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.OR_PENDING_REASON</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5493,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.SH_RATE_OFFERING_GID</t>
         </is>
       </c>
     </row>
@@ -5530,7 +5530,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.SH_RATE_GEO_GID</t>
         </is>
       </c>
     </row>
@@ -5562,7 +5562,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_XLANE_UPDATE.X_LANE_GID</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.SH_TRANSPORT_MODE_GID</t>
         </is>
       </c>
     </row>
@@ -5700,7 +5700,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.SCHEDULE_UPDATE_USER</t>
         </is>
       </c>
     </row>
@@ -5865,7 +5865,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.DOCK_DOOR</t>
         </is>
       </c>
     </row>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.LOAD_TYPE</t>
         </is>
       </c>
     </row>
@@ -6547,7 +6547,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables) - SOA_SHIPPED_QUANTITY (derived: QTY_REQUESTED - SOA_SHIPPED_QUANTITY)</t>
+          <t>Derived: QTY_REQUESTED - NBLBI_PLP.FACT_SALES_ORDERLINE_SOASHIPPEDQUANTITY_PLP.SOA_SHIPPED_QUANTITY</t>
         </is>
       </c>
     </row>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables) - SOA_SHIPPED_QUANTITY * DIM_INV_MASTER_ITEMS.X_ATTRIBUTE5 (capped at PKEQ24_CASES_REQUESTED)</t>
+          <t>NBLBI_PLP.FACT_SALES_ORDERLINE_SOASHIPPEDQUANTITY_PLP.SOA_SHIPPED_QUANTITY * DIM_INV_MASTER_ITEMS.X_ATTRIBUTE5 (capped at PKEQ24_CASES_REQUESTED)</t>
         </is>
       </c>
     </row>
@@ -6611,7 +6611,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables) - SOA_SHIPPED_QUANTITY (derived * X_ATTRIBUTE5)</t>
+          <t>Derived: PKEQ24_CASES_REQUESTED - SOA_SHIPPED_24PKEQCASES (from NBLBI_PLP.FACT_SALES_ORDERLINE_SOASHIPPEDQUANTITY_PLP.SOA_SHIPPED_QUANTITY)</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.SUPPLY_CHAIN_LOADTYPE</t>
         </is>
       </c>
     </row>
@@ -7271,7 +7271,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINESFACT_TRANSPORTATIONACTIVITY_UPDATE_PLP.SHIPMENT_PRELOAD</t>
         </is>
       </c>
     </row>
@@ -7303,7 +7303,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables) - SOA_SHIPPED_QUANTITY (capped at FULFILLLINEORDEREDQTY)</t>
+          <t>NBLBI_PLP.FACT_SALES_ORDERLINE_SOASHIPPEDQUANTITY_PLP.SOA_SHIPPED_QUANTITY (capped at FULFILLLINEORDEREDQTY)</t>
         </is>
       </c>
     </row>
@@ -7340,7 +7340,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.OREF_SCHEDULE_INSERT_USER</t>
         </is>
       </c>
     </row>
@@ -7377,7 +7377,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables)</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.WITH_DRAW_USER_FLAG</t>
         </is>
       </c>
     </row>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables) - SK_OSP_ID</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.OSP</t>
         </is>
       </c>
     </row>
@@ -7547,7 +7547,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>PLP (Plan Pro - SOLF/plp tables) - SK_MOSP_ID</t>
+          <t>NBLBI_PLP.SALESORDERLINEFACT_SHIPMENTACTIVITYFLOW_UPDATE.MOSP</t>
         </is>
       </c>
     </row>

</xml_diff>